<commit_message>
Updated plot_inputs function for seepage mode. Added a light blue derived head line for the specified head boundary lines. Added dashed lines for both head and exit face.
</commit_message>
<xml_diff>
--- a/inputs/slope/input_template_rface6.xlsx
+++ b/inputs/slope/input_template_rface6.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/cursor_projects/xslope/inputs/slope/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/inputs/slope/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2680F06C-570A-4140-8C25-98B64260E803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{761085B4-45DB-E94E-94B4-BDDB17039621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27780" yWindow="1640" windowWidth="30380" windowHeight="20300" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="6160" yWindow="1620" windowWidth="31400" windowHeight="23280" activeTab="3" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1003,7 +1003,14 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="10">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2652,6 +2659,12 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2661,6 +2674,12 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>80</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2862,6 +2881,15 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>204.3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>320</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2871,6 +2899,15 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>84</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>40</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -5655,7 +5692,7 @@
         <v>111</v>
       </c>
       <c r="C3" s="31">
-        <v>302</v>
+        <v>80</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>111</v>
@@ -5687,16 +5724,24 @@
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
+      <c r="B5" s="3">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0</v>
+      </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
+      <c r="B6" s="3">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3">
+        <v>80</v>
+      </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="H6" s="3"/>
@@ -5765,16 +5810,28 @@
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
+      <c r="B16" s="3">
+        <v>150</v>
+      </c>
+      <c r="C16" s="3">
+        <v>84</v>
+      </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
+      <c r="B17" s="3">
+        <v>204.3</v>
+      </c>
+      <c r="C17" s="3">
+        <v>40</v>
+      </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
+      <c r="B18" s="3">
+        <v>320</v>
+      </c>
+      <c r="C18" s="3">
+        <v>40</v>
+      </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" s="3"/>
@@ -6346,16 +6403,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="G22:H22"/>
     <mergeCell ref="J22:K22"/>
     <mergeCell ref="M22:N22"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6521,13 +6578,27 @@
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="4"/>
+      <c r="R4" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="S4" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="T4" s="3">
+        <v>0</v>
+      </c>
+      <c r="U4" s="3">
+        <v>1E-4</v>
+      </c>
+      <c r="V4" s="3">
+        <v>-1</v>
+      </c>
+      <c r="W4" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="X4" s="3">
+        <v>0.35</v>
+      </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
@@ -6561,13 +6632,27 @@
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-      <c r="U5" s="3"/>
-      <c r="V5" s="3"/>
-      <c r="W5" s="3"/>
-      <c r="X5" s="4"/>
+      <c r="R5" s="3">
+        <v>1</v>
+      </c>
+      <c r="S5" s="3">
+        <v>1</v>
+      </c>
+      <c r="T5" s="3">
+        <v>0</v>
+      </c>
+      <c r="U5" s="3">
+        <v>1E-4</v>
+      </c>
+      <c r="V5" s="3">
+        <v>-1</v>
+      </c>
+      <c r="W5" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="X5" s="3">
+        <v>0.35</v>
+      </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
@@ -6601,13 +6686,27 @@
       <c r="O6" s="3"/>
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
-      <c r="S6" s="3"/>
-      <c r="T6" s="3"/>
-      <c r="U6" s="3"/>
-      <c r="V6" s="3"/>
-      <c r="W6" s="3"/>
-      <c r="X6" s="4"/>
+      <c r="R6" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="S6" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="T6" s="3">
+        <v>0</v>
+      </c>
+      <c r="U6" s="3">
+        <v>1E-4</v>
+      </c>
+      <c r="V6" s="3">
+        <v>-1</v>
+      </c>
+      <c r="W6" s="3">
+        <v>500000</v>
+      </c>
+      <c r="X6" s="3">
+        <v>0.35</v>
+      </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
@@ -6999,47 +7098,52 @@
     <mergeCell ref="L2:Q2"/>
   </mergeCells>
   <conditionalFormatting sqref="E4:F15">
-    <cfRule type="expression" dxfId="8" priority="2">
+    <cfRule type="expression" dxfId="9" priority="3">
       <formula>$D4="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4:H7">
-    <cfRule type="expression" dxfId="7" priority="1">
+    <cfRule type="expression" dxfId="8" priority="2">
       <formula>$D4="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G8:J15">
-    <cfRule type="expression" dxfId="6" priority="12">
+    <cfRule type="expression" dxfId="7" priority="13">
       <formula>$D8="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I4:J7">
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="6" priority="4">
       <formula>$D4="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M4:N15">
-    <cfRule type="expression" dxfId="4" priority="10">
+    <cfRule type="expression" dxfId="5" priority="11">
       <formula>$D4="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O4:O15">
-    <cfRule type="expression" dxfId="3" priority="11">
+    <cfRule type="expression" dxfId="4" priority="12">
       <formula>$D4="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P4:Q7">
-    <cfRule type="expression" dxfId="2" priority="7">
+    <cfRule type="expression" dxfId="3" priority="8">
       <formula>$D4="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P8:Q15">
-    <cfRule type="expression" dxfId="1" priority="8">
+    <cfRule type="expression" dxfId="2" priority="9">
       <formula>$D8="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R4:V15">
-    <cfRule type="expression" dxfId="0" priority="6">
+  <conditionalFormatting sqref="R7:V15">
+    <cfRule type="expression" dxfId="1" priority="7">
+      <formula>$D7="cp"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R4:V6">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>$D4="cp"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>